<commit_message>
Show subcategories in transaction table
</commit_message>
<xml_diff>
--- a/data/transactions.xlsx
+++ b/data/transactions.xlsx
@@ -397,10 +397,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>description</v>
+      </c>
+      <c r="C1" t="str">
+        <v>category</v>
+      </c>
+      <c r="D1" t="str">
+        <v>subcategory</v>
+      </c>
+      <c r="E1" t="str">
+        <v>type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="G1" t="str">
+        <v>id</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="B2" t="str">
+        <v>test1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Food</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="F2">
+        <v>200</v>
+      </c>
+      <c r="G2">
+        <v>1788534859771</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="B3" t="str">
+        <v>1000</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Food</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3">
+        <v>1788532371567</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>